<commit_message>
Atualização automática: reajuste (16/10/2026 12:23)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/01_Bases_Originais/Reajuste/Planilha Demonstrativa -2_Reajuste - Contrato 005_CELOG-PAMALS_2025.xlsx
+++ b/Contrato 005/Dashboard/01_Bases_Originais/Reajuste/Planilha Demonstrativa -2_Reajuste - Contrato 005_CELOG-PAMALS_2025.xlsx
@@ -26,7 +26,7 @@
   <commentList>
     <comment authorId="0" ref="B71">
       <text>
-        <t xml:space="preserve">NFS-e 69 recebida em 14/10/2026. PENDENTE: descricao com competencia agosto/2026 (correto setembro/2026). Correcao/reemissao pedida a VEE ONE em 15/10/2026; atualizar o numero se for reemitida. - Wallace
+        <t xml:space="preserve">NFS-e 71 (14/10/2026), reemitida pela VEE ONE em substituicao a NFS-e 69 (competencia corrigida para setembro/2026). Enviada a COMREC para pagamento em 16/10/2026: NE 2026NE001551 R$ 117.742,58 + NE 2026NE000842 R$ 1.447.765,18.
 ======</t>
       </text>
     </comment>
@@ -4185,7 +4185,7 @@
         <v>61</v>
       </c>
       <c r="B71" s="89">
-        <v>69.0</v>
+        <v>71.0</v>
       </c>
       <c r="C71" s="88">
         <v>1565507.76</v>

</xml_diff>